<commit_message>
update raw data de portal del cliente
</commit_message>
<xml_diff>
--- a/Raw Data - 6061_OC-CR.xlsx
+++ b/Raw Data - 6061_OC-CR.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://idbg-my.sharepoint.com/personal/marcosve_iadb_org/Documents/Desktop/RawDataTemplates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mvergarc\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="468" documentId="11_F25DC773A252ABDACC104874C1D878985ADE58FB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7556C3C6-7456-4E0A-92B7-0E2773F5FA75}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D2A006-DDB0-4940-988B-C0A4FD8C0D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -731,6 +731,12 @@
     <t>{{amendmentsignatureddate}}</t>
   </si>
   <si>
+    <t>{{executionwbs}}</t>
+  </si>
+  <si>
+    <t>WBS</t>
+  </si>
+  <si>
     <t>CR-L1157</t>
   </si>
   <si>
@@ -803,6 +809,9 @@
     <t>Ninguno</t>
   </si>
   <si>
+    <t>1.1.2</t>
+  </si>
+  <si>
     <t>CR-L1157-P00003-AA</t>
   </si>
   <si>
@@ -833,6 +842,9 @@
     <t>Sustitución de 40.000 luminarias de vapor de sodio en el alumbrado público administrado por el ICE, reemplazándolas por unidades LED. Las intervenciones se focalizan en zonas semiurbanas y rurales que no han sido atendidas en fases previas, con el fin de completar la modernización del parque de iluminación nacional.</t>
   </si>
   <si>
+    <t>2026LI-000002-PROV</t>
+  </si>
+  <si>
     <t>3.1.1</t>
   </si>
   <si>
@@ -848,10 +860,7 @@
     <t>CR-L1157-P00005</t>
   </si>
   <si>
-    <t>Adquisición de transformadores elevadores</t>
-  </si>
-  <si>
-    <t>Adquisición de transformadores elevadores Modernización Ventanas Garita  </t>
+    <t>Adquisición de transformadores elevadores modernización Ventanas Garita (Incluye servicios de Supervisión y Capacitación)</t>
   </si>
   <si>
     <t>CR-L1157-P00006</t>
@@ -875,6 +884,66 @@
     <t>Adquisición de draga para limpieza del embalse</t>
   </si>
   <si>
+    <t>1.2.2</t>
+  </si>
+  <si>
+    <t>CR-L1157-P00008</t>
+  </si>
+  <si>
+    <t>Contratación de Estudios Técnicos de Proyectos de Inversión. Proyectos de almacenamiento por bombeo</t>
+  </si>
+  <si>
+    <t>Firmas Consultoras</t>
+  </si>
+  <si>
+    <t>Selección Basada en la Calidad y Costo (SBCC)</t>
+  </si>
+  <si>
+    <t>1.3.1</t>
+  </si>
+  <si>
+    <t>Estudios técnicos de proyectos de inversión desarrollados.</t>
+  </si>
+  <si>
+    <t>CR-L1157-P00009</t>
+  </si>
+  <si>
+    <t>Herramienta de modelación energética en desarrollos en cascada</t>
+  </si>
+  <si>
+    <t>1.3.2</t>
+  </si>
+  <si>
+    <t>CR-L1157-P00010</t>
+  </si>
+  <si>
+    <t>Sistemas de protección y control para subestaciones </t>
+  </si>
+  <si>
+    <t>CR-L1157-P00011-AA</t>
+  </si>
+  <si>
+    <t>Proceso adquisición equipos de AT Anillo Miravalles</t>
+  </si>
+  <si>
+    <t>2025XE-000823-00004-00001</t>
+  </si>
+  <si>
+    <t>2.1.2</t>
+  </si>
+  <si>
+    <t>CR-L1157-P00012-AA</t>
+  </si>
+  <si>
+    <t>Adquisición de componentes hilo guarda OPGW y servicio de instalación </t>
+  </si>
+  <si>
+    <t>2025XE-000940-0000400001</t>
+  </si>
+  <si>
+    <t>2.1.3</t>
+  </si>
+  <si>
     <t>Publicación del AEA</t>
   </si>
   <si>
@@ -894,6 +963,36 @@
   </si>
   <si>
     <t>Final</t>
+  </si>
+  <si>
+    <t>Publicación del Aviso de Expresión de Interés</t>
+  </si>
+  <si>
+    <t>Solicitud de Propuestas</t>
+  </si>
+  <si>
+    <t>Acta de Apertura de Propuestas (Técnica)</t>
+  </si>
+  <si>
+    <t>Reporte de Evaluación (Técnica)</t>
+  </si>
+  <si>
+    <t>Acta de Apertura de Propuestas (Financiera)</t>
+  </si>
+  <si>
+    <t>Reporte de Evaluación Final y Contrato Negociado</t>
+  </si>
+  <si>
+    <t>Notificación de Adjudicación</t>
+  </si>
+  <si>
+    <t>Se ajustó la fecha de apertura de ofertas de acuerdo al PEP del taller de arranque, por lo que se va a solicitar la No objeción del Banco, dado que se recibieron muchas aclaraciones luego de la visita de los oferentes a planta el 24 de agosto. </t>
+  </si>
+  <si>
+    <t>nbarquero@ice.go.cr</t>
+  </si>
+  <si>
+    <t>Se ajustan los plazos conforme a los acuerdos establecidos durante el Taller de Arranque.</t>
   </si>
 </sst>
 </file>
@@ -943,7 +1042,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -956,6 +1055,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -972,10 +1074,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1241,21 +1339,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:Z13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="3" width="25.77734375" customWidth="1"/>
-    <col min="4" max="5" width="150.77734375" customWidth="1"/>
-    <col min="6" max="8" width="25.77734375" customWidth="1"/>
-    <col min="9" max="9" width="50.77734375" customWidth="1"/>
-    <col min="10" max="10" width="25.77734375" customWidth="1"/>
-    <col min="11" max="12" width="25.77734375" style="3" customWidth="1"/>
-    <col min="13" max="22" width="25.77734375" customWidth="1"/>
-    <col min="23" max="23" width="50.77734375" customWidth="1"/>
-    <col min="24" max="25" width="25.77734375" customWidth="1"/>
+    <col min="1" max="3" width="25.6640625" customWidth="1"/>
+    <col min="4" max="5" width="150.6640625" customWidth="1"/>
+    <col min="6" max="8" width="25.6640625" customWidth="1"/>
+    <col min="9" max="9" width="50.6640625" customWidth="1"/>
+    <col min="10" max="10" width="25.6640625" customWidth="1"/>
+    <col min="11" max="12" width="25.6640625" style="3" customWidth="1"/>
+    <col min="13" max="22" width="25.6640625" customWidth="1"/>
+    <col min="23" max="23" width="50.6640625" customWidth="1"/>
+    <col min="24" max="25" width="25.6640625" customWidth="1"/>
+    <col min="26" max="26" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s" s="1">
         <v>127</v>
       </c>
@@ -1331,33 +1430,38 @@
       <c r="Y1" t="s" s="1">
         <v>149</v>
       </c>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z1" t="s" s="1">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B2" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D2" t="s">
+        <v>233</v>
+      </c>
+      <c r="E2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F2" t="s">
         <v>231</v>
       </c>
-      <c r="E2" t="s">
-        <v>232</v>
-      </c>
-      <c r="F2"/>
       <c r="G2"/>
       <c r="H2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="J2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="K2" t="n" s="3">
         <v>72691399.04</v>
@@ -1373,62 +1477,63 @@
         <v>0</v>
       </c>
       <c r="P2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="Q2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="R2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="S2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="T2" t="n">
         <v>1</v>
       </c>
       <c r="U2"/>
       <c r="V2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="W2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="X2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="Y2" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+      <c r="Z2"/>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="F3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="G3"/>
       <c r="H3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="J3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="K3" t="n" s="3">
         <v>2394535</v>
@@ -1444,60 +1549,63 @@
         <v>0</v>
       </c>
       <c r="P3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="Q3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="R3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="S3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="T3" t="n">
         <v>1</v>
       </c>
       <c r="U3"/>
       <c r="V3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="W3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="X3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="Y3"/>
-    </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B4" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="C4" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D4" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="E4" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="F4" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="G4"/>
       <c r="H4" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I4" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="J4" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="K4" t="n" s="3">
         <v>4721824</v>
@@ -1513,58 +1621,61 @@
         <v>0</v>
       </c>
       <c r="P4" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="Q4" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="R4" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="S4" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="T4" t="n">
         <v>1</v>
       </c>
       <c r="U4"/>
       <c r="V4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="W4" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="X4" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="Y4"/>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z4"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B5" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="C5" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D5" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="E5" t="s">
-        <v>261</v>
-      </c>
-      <c r="F5"/>
+        <v>264</v>
+      </c>
+      <c r="F5" t="s">
+        <v>265</v>
+      </c>
       <c r="G5"/>
       <c r="H5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="J5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="K5" t="n" s="3">
         <v>6920000</v>
@@ -1580,61 +1691,62 @@
         <v>0</v>
       </c>
       <c r="P5" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="Q5" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="R5" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="S5" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="T5" t="n">
         <v>1</v>
       </c>
       <c r="U5"/>
       <c r="V5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="W5" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="X5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="Y5"/>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z5"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B6" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="C6" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D6" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="E6" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F6"/>
       <c r="G6"/>
       <c r="H6" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I6" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="J6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="K6" t="n" s="3">
-        <v>4500000</v>
+        <v>4092311.58</v>
       </c>
       <c r="L6" s="3"/>
       <c r="M6" t="n">
@@ -1647,58 +1759,61 @@
         <v>0</v>
       </c>
       <c r="P6" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="Q6" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="R6" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="S6" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="T6" t="n">
         <v>1</v>
       </c>
       <c r="U6"/>
       <c r="V6" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="W6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="X6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="Y6"/>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z6" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B7" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C7" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D7" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E7" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F7"/>
       <c r="G7"/>
       <c r="H7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I7" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="J7" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="K7" t="n" s="3">
         <v>2545000</v>
@@ -1714,58 +1829,61 @@
         <v>0</v>
       </c>
       <c r="P7" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="Q7" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="R7" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="S7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="T7" t="n">
         <v>1</v>
       </c>
       <c r="U7"/>
       <c r="V7" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="W7" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="X7" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="Y7"/>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="Z7" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B8" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C8" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D8" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="E8" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F8"/>
       <c r="G8"/>
       <c r="H8" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I8" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="J8" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="K8" t="n" s="3">
         <v>1930000</v>
@@ -1781,31 +1899,372 @@
         <v>0</v>
       </c>
       <c r="P8" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="Q8" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="R8" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="S8" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="T8" t="n">
         <v>1</v>
       </c>
       <c r="U8"/>
       <c r="V8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="W8" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="X8" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y8"/>
+      <c r="Z8" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B9" t="s">
+        <v>280</v>
+      </c>
+      <c r="C9" t="s">
+        <v>232</v>
+      </c>
+      <c r="D9" t="s">
+        <v>281</v>
+      </c>
+      <c r="E9" t="s">
+        <v>281</v>
+      </c>
+      <c r="F9"/>
+      <c r="G9"/>
+      <c r="H9" t="s">
+        <v>282</v>
+      </c>
+      <c r="I9" t="s">
+        <v>283</v>
+      </c>
+      <c r="J9" t="s">
+        <v>237</v>
+      </c>
+      <c r="K9" t="n" s="3">
+        <v>250000</v>
+      </c>
+      <c r="L9" s="3"/>
+      <c r="M9" t="n">
+        <v>100</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>239</v>
+      </c>
+      <c r="R9" t="s">
+        <v>285</v>
+      </c>
+      <c r="S9" t="s">
+        <v>252</v>
+      </c>
+      <c r="T9"/>
+      <c r="U9"/>
+      <c r="V9"/>
+      <c r="W9"/>
+      <c r="X9" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y9"/>
+      <c r="Z9" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>230</v>
+      </c>
+      <c r="B10" t="s">
+        <v>286</v>
+      </c>
+      <c r="C10" t="s">
+        <v>232</v>
+      </c>
+      <c r="D10" t="s">
+        <v>287</v>
+      </c>
+      <c r="E10" t="s">
+        <v>287</v>
+      </c>
+      <c r="F10"/>
+      <c r="G10"/>
+      <c r="H10" t="s">
+        <v>282</v>
+      </c>
+      <c r="I10" t="s">
+        <v>283</v>
+      </c>
+      <c r="J10" t="s">
+        <v>237</v>
+      </c>
+      <c r="K10" t="n" s="3">
+        <v>250000</v>
+      </c>
+      <c r="L10" s="3"/>
+      <c r="M10" t="n">
+        <v>100</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="s">
+        <v>284</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>239</v>
+      </c>
+      <c r="R10" t="s">
+        <v>285</v>
+      </c>
+      <c r="S10" t="s">
+        <v>252</v>
+      </c>
+      <c r="T10"/>
+      <c r="U10"/>
+      <c r="V10"/>
+      <c r="W10"/>
+      <c r="X10" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y10"/>
+      <c r="Z10" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>230</v>
+      </c>
+      <c r="B11" t="s">
+        <v>289</v>
+      </c>
+      <c r="C11" t="s">
+        <v>232</v>
+      </c>
+      <c r="D11" t="s">
+        <v>290</v>
+      </c>
+      <c r="E11" t="s">
+        <v>290</v>
+      </c>
+      <c r="F11"/>
+      <c r="G11"/>
+      <c r="H11" t="s">
+        <v>235</v>
+      </c>
+      <c r="I11" t="s">
+        <v>236</v>
+      </c>
+      <c r="J11" t="s">
+        <v>237</v>
+      </c>
+      <c r="K11" t="n" s="3">
+        <v>36234025.69</v>
+      </c>
+      <c r="L11" s="3"/>
+      <c r="M11" t="n">
+        <v>100</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="s">
+        <v>259</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>260</v>
+      </c>
+      <c r="R11" t="s">
+        <v>261</v>
+      </c>
+      <c r="S11" t="s">
+        <v>252</v>
+      </c>
+      <c r="T11" t="n">
+        <v>3</v>
+      </c>
+      <c r="U11"/>
+      <c r="V11" t="s">
+        <v>242</v>
+      </c>
+      <c r="W11" t="s">
+        <v>243</v>
+      </c>
+      <c r="X11" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y11"/>
+      <c r="Z11" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>230</v>
+      </c>
+      <c r="B12" t="s">
+        <v>291</v>
+      </c>
+      <c r="C12" t="s">
+        <v>232</v>
+      </c>
+      <c r="D12" t="s">
+        <v>292</v>
+      </c>
+      <c r="E12" t="s">
+        <v>292</v>
+      </c>
+      <c r="F12" t="s">
+        <v>293</v>
+      </c>
+      <c r="G12"/>
+      <c r="H12" t="s">
+        <v>235</v>
+      </c>
+      <c r="I12" t="s">
+        <v>250</v>
+      </c>
+      <c r="J12" t="s">
         <v>251</v>
       </c>
-      <c r="Y8"/>
+      <c r="K12" t="n" s="3">
+        <v>3900337</v>
+      </c>
+      <c r="L12" s="3"/>
+      <c r="M12" t="n">
+        <v>100</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="s">
+        <v>259</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>260</v>
+      </c>
+      <c r="R12" t="s">
+        <v>261</v>
+      </c>
+      <c r="S12" t="s">
+        <v>252</v>
+      </c>
+      <c r="T12" t="n">
+        <v>1</v>
+      </c>
+      <c r="U12"/>
+      <c r="V12" t="s">
+        <v>242</v>
+      </c>
+      <c r="W12"/>
+      <c r="X12" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y12"/>
+      <c r="Z12" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>230</v>
+      </c>
+      <c r="B13" t="s">
+        <v>295</v>
+      </c>
+      <c r="C13" t="s">
+        <v>232</v>
+      </c>
+      <c r="D13" t="s">
+        <v>296</v>
+      </c>
+      <c r="E13" t="s">
+        <v>296</v>
+      </c>
+      <c r="F13" t="s">
+        <v>297</v>
+      </c>
+      <c r="G13"/>
+      <c r="H13" t="s">
+        <v>235</v>
+      </c>
+      <c r="I13" t="s">
+        <v>250</v>
+      </c>
+      <c r="J13" t="s">
+        <v>251</v>
+      </c>
+      <c r="K13" t="n" s="3">
+        <v>9487740.73</v>
+      </c>
+      <c r="L13" s="3"/>
+      <c r="M13" t="n">
+        <v>100</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="s">
+        <v>259</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>260</v>
+      </c>
+      <c r="R13" t="s">
+        <v>261</v>
+      </c>
+      <c r="S13" t="s">
+        <v>252</v>
+      </c>
+      <c r="T13" t="n">
+        <v>2</v>
+      </c>
+      <c r="U13"/>
+      <c r="V13" t="s">
+        <v>242</v>
+      </c>
+      <c r="W13"/>
+      <c r="X13" t="s">
+        <v>253</v>
+      </c>
+      <c r="Y13"/>
+      <c r="Z13" t="s">
+        <v>298</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1814,12 +2273,12 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51DE2F5A-B556-444D-9D4D-E87C59CE645A}">
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="25.77734375" customWidth="1"/>
-    <col min="3" max="3" width="25.77734375" style="5" customWidth="1"/>
-    <col min="4" max="5" width="25.77734375" customWidth="1"/>
+    <col min="1" max="2" width="25.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" style="5" customWidth="1"/>
+    <col min="4" max="5" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1837,6 +2296,91 @@
       </c>
       <c r="E1" t="s" s="1">
         <v>226</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>231</v>
+      </c>
+      <c r="B2" t="s">
+        <v>233</v>
+      </c>
+      <c r="C2" t="n" s="5">
+        <v>46269</v>
+      </c>
+      <c r="D2" t="s">
+        <v>313</v>
+      </c>
+      <c r="E2" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B3" t="s">
+        <v>263</v>
+      </c>
+      <c r="C3" t="n" s="5">
+        <v>46269</v>
+      </c>
+      <c r="D3" t="s">
+        <v>315</v>
+      </c>
+      <c r="E3" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>270</v>
+      </c>
+      <c r="B4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C4" t="n" s="5">
+        <v>46269</v>
+      </c>
+      <c r="D4" t="s">
+        <v>315</v>
+      </c>
+      <c r="E4" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>272</v>
+      </c>
+      <c r="B5" t="s">
+        <v>273</v>
+      </c>
+      <c r="C5" t="n" s="5">
+        <v>46269</v>
+      </c>
+      <c r="D5" t="s">
+        <v>315</v>
+      </c>
+      <c r="E5" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>277</v>
+      </c>
+      <c r="B6" t="s">
+        <v>278</v>
+      </c>
+      <c r="C6" t="n" s="5">
+        <v>46269</v>
+      </c>
+      <c r="D6" t="s">
+        <v>315</v>
+      </c>
+      <c r="E6" t="s">
+        <v>314</v>
       </c>
     </row>
   </sheetData>
@@ -1846,15 +2390,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA70B816-A7E8-478F-96D4-061C9871C9B8}">
-  <dimension ref="A1:K30"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.77734375" customWidth="1"/>
-    <col min="2" max="2" width="150.77734375" customWidth="1"/>
-    <col min="3" max="4" width="25.77734375" customWidth="1"/>
-    <col min="5" max="5" width="50.77734375" customWidth="1"/>
-    <col min="6" max="6" width="25.77734375" customWidth="1"/>
-    <col min="7" max="11" width="25.77734375" style="5" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="150.6640625" customWidth="1"/>
+    <col min="3" max="4" width="25.6640625" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" customWidth="1"/>
+    <col min="6" max="6" width="25.6640625" customWidth="1"/>
+    <col min="7" max="11" width="25.6640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1894,22 +2438,22 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F2" t="s">
-        <v>276</v>
+        <v>299</v>
       </c>
       <c r="G2" t="n" s="5">
         <v>46227</v>
@@ -1925,28 +2469,28 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F3" t="s">
-        <v>277</v>
+        <v>300</v>
       </c>
       <c r="G3" t="n" s="5">
         <v>46352</v>
       </c>
       <c r="H3" t="n" s="5">
-        <v>46352</v>
+        <v>46357</v>
       </c>
       <c r="I3" s="5"/>
       <c r="J3" s="5"/>
@@ -1954,28 +2498,28 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B4" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C4" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E4" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F4" t="s">
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="G4" t="n" s="5">
         <v>46468</v>
       </c>
       <c r="H4" t="n" s="5">
-        <v>46468</v>
+        <v>46471</v>
       </c>
       <c r="I4" s="5"/>
       <c r="J4" s="5"/>
@@ -1983,28 +2527,28 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D5" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F5" t="s">
-        <v>279</v>
+        <v>302</v>
       </c>
       <c r="G5" t="n" s="5">
         <v>46505</v>
       </c>
       <c r="H5" t="n" s="5">
-        <v>46505</v>
+        <v>46510</v>
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
@@ -2012,28 +2556,28 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B6" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C6" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D6" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F6" t="s">
-        <v>280</v>
+        <v>303</v>
       </c>
       <c r="G6" t="n" s="5">
         <v>46549</v>
       </c>
       <c r="H6" t="n" s="5">
-        <v>46549</v>
+        <v>46554</v>
       </c>
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
@@ -2041,52 +2585,54 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B7" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C7" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D7" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E7" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F7" t="s">
-        <v>281</v>
+        <v>304</v>
       </c>
       <c r="G7" t="n" s="5">
         <v>45695</v>
       </c>
       <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
+      <c r="I7" t="n" s="5">
+        <v>46287</v>
+      </c>
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B8" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C8" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D8" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E8" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F8" t="s">
-        <v>282</v>
+        <v>305</v>
       </c>
       <c r="G8" t="n" s="5">
-        <v>46056</v>
+        <v>46055</v>
       </c>
       <c r="H8" s="5"/>
       <c r="I8" s="5"/>
@@ -2095,22 +2641,22 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B9" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C9" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D9" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E9" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F9" t="s">
-        <v>281</v>
+        <v>304</v>
       </c>
       <c r="G9" t="n" s="5">
         <v>45638</v>
@@ -2122,22 +2668,22 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B10" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C10" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D10" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E10" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="F10" t="s">
-        <v>282</v>
+        <v>305</v>
       </c>
       <c r="G10" t="n" s="5">
         <v>45971</v>
@@ -2149,160 +2695,172 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B11" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C11" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D11" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E11" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F11" t="s">
-        <v>276</v>
+        <v>299</v>
       </c>
       <c r="G11" t="n" s="5">
         <v>46227</v>
       </c>
-      <c r="H11" s="5"/>
-      <c r="I11" s="5"/>
+      <c r="H11" t="n" s="5">
+        <v>46227</v>
+      </c>
+      <c r="I11" t="n" s="5">
+        <v>46258</v>
+      </c>
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B12" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C12" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D12" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E12" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F12" t="s">
-        <v>277</v>
+        <v>300</v>
       </c>
       <c r="G12" t="n" s="5">
         <v>46273</v>
       </c>
-      <c r="H12" s="5"/>
+      <c r="H12" t="n" s="5">
+        <v>46273</v>
+      </c>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B13" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C13" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D13" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E13" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F13" t="s">
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="G13" t="n" s="5">
         <v>46367</v>
       </c>
-      <c r="H13" s="5"/>
+      <c r="H13" t="n" s="5">
+        <v>46367</v>
+      </c>
       <c r="I13" s="5"/>
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B14" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C14" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D14" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E14" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F14" t="s">
-        <v>279</v>
+        <v>302</v>
       </c>
       <c r="G14" t="n" s="5">
         <v>46399</v>
       </c>
-      <c r="H14" s="5"/>
+      <c r="H14" t="n" s="5">
+        <v>46399</v>
+      </c>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B15" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="C15" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D15" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E15" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F15" t="s">
-        <v>280</v>
+        <v>303</v>
       </c>
       <c r="G15" t="n" s="5">
         <v>46457</v>
       </c>
-      <c r="H15" s="5"/>
+      <c r="H15" t="n" s="5">
+        <v>46457</v>
+      </c>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B16" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C16" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D16" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E16" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F16" t="s">
-        <v>276</v>
+        <v>299</v>
       </c>
       <c r="G16" t="n" s="5">
-        <v>46342</v>
+        <v>46325</v>
       </c>
       <c r="H16" s="5"/>
       <c r="I16" s="5"/>
@@ -2311,25 +2869,25 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B17" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C17" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D17" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E17" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F17" t="s">
-        <v>277</v>
+        <v>300</v>
       </c>
       <c r="G17" t="n" s="5">
-        <v>46465</v>
+        <v>46450</v>
       </c>
       <c r="H17" s="5"/>
       <c r="I17" s="5"/>
@@ -2338,25 +2896,25 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B18" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C18" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D18" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E18" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F18" t="s">
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="G18" t="n" s="5">
-        <v>46561</v>
+        <v>46546</v>
       </c>
       <c r="H18" s="5"/>
       <c r="I18" s="5"/>
@@ -2365,25 +2923,25 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B19" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C19" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D19" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E19" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F19" t="s">
-        <v>279</v>
+        <v>302</v>
       </c>
       <c r="G19" t="n" s="5">
-        <v>46591</v>
+        <v>46576</v>
       </c>
       <c r="H19" s="5"/>
       <c r="I19" s="5"/>
@@ -2392,25 +2950,25 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>266</v>
+        <v>270</v>
       </c>
       <c r="B20" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="C20" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D20" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E20" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F20" t="s">
-        <v>280</v>
+        <v>303</v>
       </c>
       <c r="G20" t="n" s="5">
-        <v>46637</v>
+        <v>46622</v>
       </c>
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
@@ -2419,25 +2977,25 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B21" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C21" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D21" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E21" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F21" t="s">
-        <v>276</v>
+        <v>299</v>
       </c>
       <c r="G21" t="n" s="5">
-        <v>46398</v>
+        <v>46413</v>
       </c>
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
@@ -2446,25 +3004,25 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B22" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C22" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D22" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E22" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F22" t="s">
-        <v>277</v>
+        <v>300</v>
       </c>
       <c r="G22" t="n" s="5">
-        <v>46521</v>
+        <v>46538</v>
       </c>
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
@@ -2473,25 +3031,25 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B23" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C23" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D23" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E23" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F23" t="s">
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="G23" t="n" s="5">
-        <v>46640</v>
+        <v>46657</v>
       </c>
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
@@ -2500,25 +3058,25 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B24" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C24" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D24" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E24" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F24" t="s">
-        <v>279</v>
+        <v>302</v>
       </c>
       <c r="G24" t="n" s="5">
-        <v>46672</v>
+        <v>46687</v>
       </c>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
@@ -2527,25 +3085,25 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B25" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="C25" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D25" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E25" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F25" t="s">
-        <v>280</v>
+        <v>303</v>
       </c>
       <c r="G25" t="n" s="5">
-        <v>46716</v>
+        <v>46731</v>
       </c>
       <c r="H25" s="5"/>
       <c r="I25" s="5"/>
@@ -2554,25 +3112,25 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B26" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C26" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D26" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E26" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F26" t="s">
-        <v>276</v>
+        <v>299</v>
       </c>
       <c r="G26" t="n" s="5">
-        <v>46492</v>
+        <v>46497</v>
       </c>
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
@@ -2581,25 +3139,25 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B27" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C27" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D27" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E27" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F27" t="s">
-        <v>277</v>
+        <v>300</v>
       </c>
       <c r="G27" t="n" s="5">
-        <v>46679</v>
+        <v>46682</v>
       </c>
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
@@ -2608,25 +3166,25 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B28" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C28" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D28" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E28" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F28" t="s">
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="G28" t="n" s="5">
-        <v>46758</v>
+        <v>46763</v>
       </c>
       <c r="H28" s="5"/>
       <c r="I28" s="5"/>
@@ -2635,25 +3193,25 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B29" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C29" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D29" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E29" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F29" t="s">
-        <v>279</v>
+        <v>302</v>
       </c>
       <c r="G29" t="n" s="5">
-        <v>46790</v>
+        <v>46793</v>
       </c>
       <c r="H29" s="5"/>
       <c r="I29" s="5"/>
@@ -2662,30 +3220,705 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B30" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="C30" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D30" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E30" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F30" t="s">
-        <v>280</v>
+        <v>303</v>
       </c>
       <c r="G30" t="n" s="5">
-        <v>46834</v>
+        <v>46839</v>
       </c>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
       <c r="K30" s="5"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>280</v>
+      </c>
+      <c r="B31" t="s">
+        <v>281</v>
+      </c>
+      <c r="C31" t="s">
+        <v>282</v>
+      </c>
+      <c r="D31" t="s">
+        <v>283</v>
+      </c>
+      <c r="E31" t="s">
+        <v>237</v>
+      </c>
+      <c r="F31" t="s">
+        <v>306</v>
+      </c>
+      <c r="G31" t="n" s="5">
+        <v>46449</v>
+      </c>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>280</v>
+      </c>
+      <c r="B32" t="s">
+        <v>281</v>
+      </c>
+      <c r="C32" t="s">
+        <v>282</v>
+      </c>
+      <c r="D32" t="s">
+        <v>283</v>
+      </c>
+      <c r="E32" t="s">
+        <v>237</v>
+      </c>
+      <c r="F32" t="s">
+        <v>307</v>
+      </c>
+      <c r="G32" t="n" s="5">
+        <v>46524</v>
+      </c>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>280</v>
+      </c>
+      <c r="B33" t="s">
+        <v>281</v>
+      </c>
+      <c r="C33" t="s">
+        <v>282</v>
+      </c>
+      <c r="D33" t="s">
+        <v>283</v>
+      </c>
+      <c r="E33" t="s">
+        <v>237</v>
+      </c>
+      <c r="F33" t="s">
+        <v>308</v>
+      </c>
+      <c r="G33" t="n" s="5">
+        <v>46553</v>
+      </c>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>280</v>
+      </c>
+      <c r="B34" t="s">
+        <v>281</v>
+      </c>
+      <c r="C34" t="s">
+        <v>282</v>
+      </c>
+      <c r="D34" t="s">
+        <v>283</v>
+      </c>
+      <c r="E34" t="s">
+        <v>237</v>
+      </c>
+      <c r="F34" t="s">
+        <v>309</v>
+      </c>
+      <c r="G34" t="n" s="5">
+        <v>46588</v>
+      </c>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>280</v>
+      </c>
+      <c r="B35" t="s">
+        <v>281</v>
+      </c>
+      <c r="C35" t="s">
+        <v>282</v>
+      </c>
+      <c r="D35" t="s">
+        <v>283</v>
+      </c>
+      <c r="E35" t="s">
+        <v>237</v>
+      </c>
+      <c r="F35" t="s">
+        <v>310</v>
+      </c>
+      <c r="G35" t="n" s="5">
+        <v>46602</v>
+      </c>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>280</v>
+      </c>
+      <c r="B36" t="s">
+        <v>281</v>
+      </c>
+      <c r="C36" t="s">
+        <v>282</v>
+      </c>
+      <c r="D36" t="s">
+        <v>283</v>
+      </c>
+      <c r="E36" t="s">
+        <v>237</v>
+      </c>
+      <c r="F36" t="s">
+        <v>311</v>
+      </c>
+      <c r="G36" t="n" s="5">
+        <v>46637</v>
+      </c>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5"/>
+      <c r="J36" s="5"/>
+      <c r="K36" s="5"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>280</v>
+      </c>
+      <c r="B37" t="s">
+        <v>281</v>
+      </c>
+      <c r="C37" t="s">
+        <v>282</v>
+      </c>
+      <c r="D37" t="s">
+        <v>283</v>
+      </c>
+      <c r="E37" t="s">
+        <v>237</v>
+      </c>
+      <c r="F37" t="s">
+        <v>312</v>
+      </c>
+      <c r="G37" t="n" s="5">
+        <v>46651</v>
+      </c>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>280</v>
+      </c>
+      <c r="B38" t="s">
+        <v>281</v>
+      </c>
+      <c r="C38" t="s">
+        <v>282</v>
+      </c>
+      <c r="D38" t="s">
+        <v>283</v>
+      </c>
+      <c r="E38" t="s">
+        <v>237</v>
+      </c>
+      <c r="F38" t="s">
+        <v>303</v>
+      </c>
+      <c r="G38" t="n" s="5">
+        <v>46695</v>
+      </c>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>286</v>
+      </c>
+      <c r="B39" t="s">
+        <v>287</v>
+      </c>
+      <c r="C39" t="s">
+        <v>282</v>
+      </c>
+      <c r="D39" t="s">
+        <v>283</v>
+      </c>
+      <c r="E39" t="s">
+        <v>237</v>
+      </c>
+      <c r="F39" t="s">
+        <v>306</v>
+      </c>
+      <c r="G39" t="n" s="5">
+        <v>46449</v>
+      </c>
+      <c r="H39" s="5"/>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5"/>
+      <c r="K39" s="5"/>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>286</v>
+      </c>
+      <c r="B40" t="s">
+        <v>287</v>
+      </c>
+      <c r="C40" t="s">
+        <v>282</v>
+      </c>
+      <c r="D40" t="s">
+        <v>283</v>
+      </c>
+      <c r="E40" t="s">
+        <v>237</v>
+      </c>
+      <c r="F40" t="s">
+        <v>307</v>
+      </c>
+      <c r="G40" t="n" s="5">
+        <v>46524</v>
+      </c>
+      <c r="H40" s="5"/>
+      <c r="I40" s="5"/>
+      <c r="J40" s="5"/>
+      <c r="K40" s="5"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>286</v>
+      </c>
+      <c r="B41" t="s">
+        <v>287</v>
+      </c>
+      <c r="C41" t="s">
+        <v>282</v>
+      </c>
+      <c r="D41" t="s">
+        <v>283</v>
+      </c>
+      <c r="E41" t="s">
+        <v>237</v>
+      </c>
+      <c r="F41" t="s">
+        <v>308</v>
+      </c>
+      <c r="G41" t="n" s="5">
+        <v>46553</v>
+      </c>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="K41" s="5"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>286</v>
+      </c>
+      <c r="B42" t="s">
+        <v>287</v>
+      </c>
+      <c r="C42" t="s">
+        <v>282</v>
+      </c>
+      <c r="D42" t="s">
+        <v>283</v>
+      </c>
+      <c r="E42" t="s">
+        <v>237</v>
+      </c>
+      <c r="F42" t="s">
+        <v>309</v>
+      </c>
+      <c r="G42" t="n" s="5">
+        <v>46588</v>
+      </c>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="K42" s="5"/>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>286</v>
+      </c>
+      <c r="B43" t="s">
+        <v>287</v>
+      </c>
+      <c r="C43" t="s">
+        <v>282</v>
+      </c>
+      <c r="D43" t="s">
+        <v>283</v>
+      </c>
+      <c r="E43" t="s">
+        <v>237</v>
+      </c>
+      <c r="F43" t="s">
+        <v>310</v>
+      </c>
+      <c r="G43" t="n" s="5">
+        <v>46602</v>
+      </c>
+      <c r="H43" s="5"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="K43" s="5"/>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>286</v>
+      </c>
+      <c r="B44" t="s">
+        <v>287</v>
+      </c>
+      <c r="C44" t="s">
+        <v>282</v>
+      </c>
+      <c r="D44" t="s">
+        <v>283</v>
+      </c>
+      <c r="E44" t="s">
+        <v>237</v>
+      </c>
+      <c r="F44" t="s">
+        <v>311</v>
+      </c>
+      <c r="G44" t="n" s="5">
+        <v>46637</v>
+      </c>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="K44" s="5"/>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>286</v>
+      </c>
+      <c r="B45" t="s">
+        <v>287</v>
+      </c>
+      <c r="C45" t="s">
+        <v>282</v>
+      </c>
+      <c r="D45" t="s">
+        <v>283</v>
+      </c>
+      <c r="E45" t="s">
+        <v>237</v>
+      </c>
+      <c r="F45" t="s">
+        <v>312</v>
+      </c>
+      <c r="G45" t="n" s="5">
+        <v>46651</v>
+      </c>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="K45" s="5"/>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>286</v>
+      </c>
+      <c r="B46" t="s">
+        <v>287</v>
+      </c>
+      <c r="C46" t="s">
+        <v>282</v>
+      </c>
+      <c r="D46" t="s">
+        <v>283</v>
+      </c>
+      <c r="E46" t="s">
+        <v>237</v>
+      </c>
+      <c r="F46" t="s">
+        <v>303</v>
+      </c>
+      <c r="G46" t="n" s="5">
+        <v>46695</v>
+      </c>
+      <c r="H46" s="5"/>
+      <c r="I46" s="5"/>
+      <c r="J46" s="5"/>
+      <c r="K46" s="5"/>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>289</v>
+      </c>
+      <c r="B47" t="s">
+        <v>290</v>
+      </c>
+      <c r="C47" t="s">
+        <v>235</v>
+      </c>
+      <c r="D47" t="s">
+        <v>236</v>
+      </c>
+      <c r="E47" t="s">
+        <v>237</v>
+      </c>
+      <c r="F47" t="s">
+        <v>299</v>
+      </c>
+      <c r="G47" t="n" s="5">
+        <v>46492</v>
+      </c>
+      <c r="H47" s="5"/>
+      <c r="I47" s="5"/>
+      <c r="J47" s="5"/>
+      <c r="K47" s="5"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>289</v>
+      </c>
+      <c r="B48" t="s">
+        <v>290</v>
+      </c>
+      <c r="C48" t="s">
+        <v>235</v>
+      </c>
+      <c r="D48" t="s">
+        <v>236</v>
+      </c>
+      <c r="E48" t="s">
+        <v>237</v>
+      </c>
+      <c r="F48" t="s">
+        <v>300</v>
+      </c>
+      <c r="G48" t="n" s="5">
+        <v>46617</v>
+      </c>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
+      <c r="K48" s="5"/>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>289</v>
+      </c>
+      <c r="B49" t="s">
+        <v>290</v>
+      </c>
+      <c r="C49" t="s">
+        <v>235</v>
+      </c>
+      <c r="D49" t="s">
+        <v>236</v>
+      </c>
+      <c r="E49" t="s">
+        <v>237</v>
+      </c>
+      <c r="F49" t="s">
+        <v>301</v>
+      </c>
+      <c r="G49" t="n" s="5">
+        <v>46728</v>
+      </c>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>289</v>
+      </c>
+      <c r="B50" t="s">
+        <v>290</v>
+      </c>
+      <c r="C50" t="s">
+        <v>235</v>
+      </c>
+      <c r="D50" t="s">
+        <v>236</v>
+      </c>
+      <c r="E50" t="s">
+        <v>237</v>
+      </c>
+      <c r="F50" t="s">
+        <v>302</v>
+      </c>
+      <c r="G50" t="n" s="5">
+        <v>46758</v>
+      </c>
+      <c r="H50" s="5"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="5"/>
+      <c r="K50" s="5"/>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>289</v>
+      </c>
+      <c r="B51" t="s">
+        <v>290</v>
+      </c>
+      <c r="C51" t="s">
+        <v>235</v>
+      </c>
+      <c r="D51" t="s">
+        <v>236</v>
+      </c>
+      <c r="E51" t="s">
+        <v>237</v>
+      </c>
+      <c r="F51" t="s">
+        <v>303</v>
+      </c>
+      <c r="G51" t="n" s="5">
+        <v>46776</v>
+      </c>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>291</v>
+      </c>
+      <c r="B52" t="s">
+        <v>292</v>
+      </c>
+      <c r="C52" t="s">
+        <v>235</v>
+      </c>
+      <c r="D52" t="s">
+        <v>250</v>
+      </c>
+      <c r="E52" t="s">
+        <v>251</v>
+      </c>
+      <c r="F52" t="s">
+        <v>304</v>
+      </c>
+      <c r="G52" t="n" s="5">
+        <v>46287</v>
+      </c>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="5"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>291</v>
+      </c>
+      <c r="B53" t="s">
+        <v>292</v>
+      </c>
+      <c r="C53" t="s">
+        <v>235</v>
+      </c>
+      <c r="D53" t="s">
+        <v>250</v>
+      </c>
+      <c r="E53" t="s">
+        <v>251</v>
+      </c>
+      <c r="F53" t="s">
+        <v>305</v>
+      </c>
+      <c r="G53" t="n" s="5">
+        <v>46288</v>
+      </c>
+      <c r="H53" s="5"/>
+      <c r="I53" s="5"/>
+      <c r="J53" s="5"/>
+      <c r="K53" s="5"/>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>295</v>
+      </c>
+      <c r="B54" t="s">
+        <v>296</v>
+      </c>
+      <c r="C54" t="s">
+        <v>235</v>
+      </c>
+      <c r="D54" t="s">
+        <v>250</v>
+      </c>
+      <c r="E54" t="s">
+        <v>251</v>
+      </c>
+      <c r="F54" t="s">
+        <v>304</v>
+      </c>
+      <c r="G54" t="n" s="5">
+        <v>46287</v>
+      </c>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="5"/>
+      <c r="K54" s="5"/>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>295</v>
+      </c>
+      <c r="B55" t="s">
+        <v>296</v>
+      </c>
+      <c r="C55" t="s">
+        <v>235</v>
+      </c>
+      <c r="D55" t="s">
+        <v>250</v>
+      </c>
+      <c r="E55" t="s">
+        <v>251</v>
+      </c>
+      <c r="F55" t="s">
+        <v>305</v>
+      </c>
+      <c r="G55" t="n" s="5">
+        <v>46288</v>
+      </c>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="5"/>
+      <c r="K55" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2695,13 +3928,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0017DABE-EE5D-40E5-AE1B-EB23E2085E81}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.77734375" customWidth="1"/>
-    <col min="2" max="2" width="150.77734375" customWidth="1"/>
-    <col min="3" max="5" width="25.77734375" customWidth="1"/>
-    <col min="6" max="6" width="25.77734375" style="3" customWidth="1"/>
-    <col min="7" max="12" width="25.77734375" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="150.6640625" customWidth="1"/>
+    <col min="3" max="5" width="25.6640625" customWidth="1"/>
+    <col min="6" max="6" width="25.6640625" style="3" customWidth="1"/>
+    <col min="7" max="12" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2750,15 +3983,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{781E74A2-A435-469D-8C02-4E4DCC83A8A8}">
   <dimension ref="A1:X1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="25.77734375" customWidth="1"/>
-    <col min="3" max="3" width="50.77734375" customWidth="1"/>
-    <col min="4" max="4" width="100.77734375" customWidth="1"/>
-    <col min="5" max="7" width="25.77734375" customWidth="1"/>
-    <col min="8" max="10" width="25.77734375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="25.77734375" style="3" customWidth="1"/>
-    <col min="12" max="24" width="25.77734375" customWidth="1"/>
+    <col min="1" max="2" width="25.6640625" customWidth="1"/>
+    <col min="3" max="3" width="50.6640625" customWidth="1"/>
+    <col min="4" max="4" width="100.6640625" customWidth="1"/>
+    <col min="5" max="7" width="25.6640625" customWidth="1"/>
+    <col min="8" max="10" width="25.6640625" style="5" customWidth="1"/>
+    <col min="11" max="11" width="25.6640625" style="3" customWidth="1"/>
+    <col min="12" max="24" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2843,13 +4076,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BBD02627-0AF2-4D0D-918E-F5CC976075FC}">
   <dimension ref="A1:T1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="25.77734375" customWidth="1"/>
-    <col min="3" max="3" width="50.77734375" customWidth="1"/>
-    <col min="4" max="5" width="25.77734375" customWidth="1"/>
-    <col min="6" max="17" width="25.77734375" style="3" customWidth="1"/>
-    <col min="18" max="20" width="25.77734375" style="5" customWidth="1"/>
+    <col min="1" max="2" width="25.6640625" customWidth="1"/>
+    <col min="3" max="3" width="50.6640625" customWidth="1"/>
+    <col min="4" max="5" width="25.6640625" customWidth="1"/>
+    <col min="6" max="17" width="25.6640625" style="3" customWidth="1"/>
+    <col min="18" max="20" width="25.6640625" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2922,12 +4155,12 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1EB3EA1-AA35-477F-A30B-FD77D094C1DA}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="4" width="25.77734375" customWidth="1"/>
-    <col min="5" max="5" width="50.77734375" customWidth="1"/>
-    <col min="6" max="6" width="25.77734375" customWidth="1"/>
-    <col min="7" max="12" width="25.77734375" style="3" customWidth="1"/>
+    <col min="1" max="4" width="25.6640625" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" customWidth="1"/>
+    <col min="6" max="6" width="25.6640625" customWidth="1"/>
+    <col min="7" max="12" width="25.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -2976,13 +4209,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B28CE9BD-E06B-4C94-8DA6-3854F70D54EC}">
   <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="4" width="25.77734375" customWidth="1"/>
-    <col min="5" max="5" width="50.77734375" customWidth="1"/>
-    <col min="6" max="6" width="25.77734375" customWidth="1"/>
-    <col min="7" max="9" width="25.77734375" style="3" customWidth="1"/>
-    <col min="10" max="11" width="25.77734375" customWidth="1"/>
+    <col min="1" max="4" width="25.6640625" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" customWidth="1"/>
+    <col min="6" max="6" width="25.6640625" customWidth="1"/>
+    <col min="7" max="9" width="25.6640625" style="3" customWidth="1"/>
+    <col min="10" max="11" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3028,13 +4261,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B33DAD8E-9201-4591-822B-ACD4E128F28B}">
   <dimension ref="A1:L1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="4" width="25.77734375" customWidth="1"/>
-    <col min="5" max="5" width="50.77734375" customWidth="1"/>
-    <col min="6" max="7" width="25.77734375" customWidth="1"/>
-    <col min="8" max="11" width="25.77734375" style="3" customWidth="1"/>
-    <col min="12" max="12" width="25.77734375" customWidth="1"/>
+    <col min="1" max="4" width="25.6640625" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" customWidth="1"/>
+    <col min="6" max="7" width="25.6640625" customWidth="1"/>
+    <col min="8" max="11" width="25.6640625" style="3" customWidth="1"/>
+    <col min="12" max="12" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -3083,11 +4316,11 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD412CD5-A879-46B1-85BB-1CD96FB59134}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="25.77734375" customWidth="1"/>
-    <col min="3" max="3" width="25.77734375" style="5" customWidth="1"/>
-    <col min="4" max="5" width="25.77734375" customWidth="1"/>
+    <col min="1" max="2" width="25.6640625" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" style="5" customWidth="1"/>
+    <col min="4" max="5" width="25.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>